<commit_message>
feat(perf): integrate baseline load test metrics and configuration
</commit_message>
<xml_diff>
--- a/unified-reports/unified-summary.xlsx
+++ b/unified-reports/unified-summary.xlsx
@@ -29,7 +29,7 @@
     <t>Execution Date:</t>
   </si>
   <si>
-    <t>2026-06-23 10:04:49 UTC</t>
+    <t>2026-06-23 11:01:51 UTC</t>
   </si>
   <si>
     <t>Branch:</t>
@@ -6016,7 +6016,7 @@
         <v>24</v>
       </c>
       <c r="B12">
-        <v>1000</v>
+        <v>7200</v>
       </c>
       <c r="C12" t="s">
         <v>21</v>

</xml_diff>